<commit_message>
RF SEASONAL: drop years 2022/2024/2026, blank single-0s again
Per sirichai: revert yesterday's expansion. Removed the three inserted
rows from the template (back to exactly 4 data rows 2025/2023/2021/2020
+ TOTAL, formulas fixed), reverted RF_SEASONAL_YEARS/YEAR_ROW, and
restored the blank-on-zero write (except TOTAL) for both the Excel sheet
and the dashboard table.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/(HAL)Stock form.xlsx
+++ b/(HAL)Stock form.xlsx
@@ -6706,8 +6706,8 @@
   <mergeCells count="46">
     <mergeCell ref="V55:W55"/>
     <mergeCell ref="W59:AO59"/>
+    <mergeCell ref="AG2:AL2"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="AG2:AL2"/>
     <mergeCell ref="A2:B3"/>
     <mergeCell ref="W58:AO58"/>
     <mergeCell ref="I43:K43"/>
@@ -6854,7 +6854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.15" customHeight="1"/>
   <cols>
     <col width="5.75" bestFit="1" customWidth="1" style="96" min="1" max="1"/>
@@ -6978,153 +6978,106 @@
       <c r="M3" s="120" t="n"/>
     </row>
     <row r="4" ht="16.15" customHeight="1">
-      <c r="A4" s="121" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B4" s="122" t="n"/>
-      <c r="C4" s="122" t="n"/>
-      <c r="D4" s="122" t="n"/>
+      <c r="A4" s="122" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B4" s="123" t="n"/>
+      <c r="C4" s="123" t="n"/>
+      <c r="D4" s="123" t="n"/>
       <c r="E4" s="118" t="n"/>
       <c r="F4" s="122" t="n">
-        <v>2026</v>
-      </c>
-      <c r="G4" s="122" t="n"/>
-      <c r="H4" s="122" t="n"/>
-      <c r="I4" s="122" t="n"/>
+        <v>2025</v>
+      </c>
+      <c r="G4" s="123" t="n"/>
+      <c r="H4" s="123" t="n"/>
+      <c r="I4" s="123" t="n"/>
       <c r="J4" s="120" t="n"/>
       <c r="K4" s="120" t="n"/>
       <c r="L4" s="120" t="n"/>
       <c r="M4" s="120" t="n"/>
     </row>
     <row r="5" ht="16.15" customHeight="1">
-      <c r="A5" s="122" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B5" s="123" t="n"/>
-      <c r="C5" s="123" t="n"/>
-      <c r="D5" s="123" t="n"/>
-      <c r="E5" s="118" t="n"/>
-      <c r="F5" s="122" t="n">
-        <v>2025</v>
-      </c>
-      <c r="G5" s="123" t="n"/>
-      <c r="H5" s="123" t="n"/>
-      <c r="I5" s="123" t="n"/>
-      <c r="J5" s="120" t="n"/>
-      <c r="K5" s="120" t="n"/>
-      <c r="L5" s="120" t="n"/>
-      <c r="M5" s="120" t="n"/>
+      <c r="A5" s="124" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B5" s="125" t="n"/>
+      <c r="C5" s="125" t="n"/>
+      <c r="D5" s="125" t="n"/>
+      <c r="E5" s="111" t="n"/>
+      <c r="F5" s="124" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G5" s="125" t="n"/>
+      <c r="H5" s="125" t="n"/>
+      <c r="I5" s="125" t="n"/>
     </row>
     <row r="6" ht="16.15" customHeight="1">
-      <c r="A6" s="122" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B6" s="123" t="n"/>
-      <c r="C6" s="123" t="n"/>
-      <c r="D6" s="123" t="n"/>
-      <c r="E6" s="118" t="n"/>
-      <c r="F6" s="122" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G6" s="123" t="n"/>
-      <c r="H6" s="123" t="n"/>
-      <c r="I6" s="123" t="n"/>
+      <c r="A6" s="124" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B6" s="125" t="n"/>
+      <c r="C6" s="125" t="n"/>
+      <c r="D6" s="125" t="n"/>
+      <c r="F6" s="124" t="n">
+        <v>2021</v>
+      </c>
+      <c r="G6" s="125" t="n"/>
+      <c r="H6" s="125" t="n"/>
+      <c r="I6" s="125" t="n"/>
     </row>
     <row r="7" ht="16.15" customHeight="1">
       <c r="A7" s="124" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="B7" s="125" t="n"/>
       <c r="C7" s="125" t="n"/>
       <c r="D7" s="125" t="n"/>
-      <c r="E7" s="111" t="n"/>
       <c r="F7" s="124" t="n">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="G7" s="125" t="n"/>
       <c r="H7" s="125" t="n"/>
       <c r="I7" s="125" t="n"/>
     </row>
     <row r="8" ht="16.15" customHeight="1" thickBot="1">
-      <c r="A8" s="124" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B8" s="125" t="n"/>
-      <c r="C8" s="125" t="n"/>
-      <c r="D8" s="125" t="n"/>
-      <c r="F8" s="124" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G8" s="125" t="n"/>
-      <c r="H8" s="125" t="n"/>
-      <c r="I8" s="125" t="n"/>
-    </row>
-    <row r="9" ht="16.15" customHeight="1" thickTop="1">
-      <c r="A9" s="124" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B9" s="125" t="n"/>
-      <c r="C9" s="125" t="n"/>
-      <c r="D9" s="125" t="n"/>
-      <c r="F9" s="124" t="n">
-        <v>2021</v>
-      </c>
-      <c r="G9" s="125" t="n"/>
-      <c r="H9" s="125" t="n"/>
-      <c r="I9" s="125" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="124" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B10" s="125" t="n"/>
-      <c r="C10" s="125" t="n"/>
-      <c r="D10" s="125" t="n"/>
-      <c r="F10" s="124" t="n">
-        <v>2020</v>
-      </c>
-      <c r="G10" s="125" t="n"/>
-      <c r="H10" s="125" t="n"/>
-      <c r="I10" s="125" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="126" t="inlineStr">
+      <c r="A8" s="126" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="127">
-        <f>SUM(B4:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="127">
-        <f>SUM(C4:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="127">
-        <f>SUM(D4:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="128" t="n"/>
-      <c r="F11" s="126" t="inlineStr">
+      <c r="B8" s="127">
+        <f>SUM(B4:B7)</f>
+        <v/>
+      </c>
+      <c r="C8" s="127">
+        <f>SUM(C4:C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="127">
+        <f>SUM(D4:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="128" t="n"/>
+      <c r="F8" s="126" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="G11" s="127">
-        <f>SUM(G4:G10)</f>
-        <v/>
-      </c>
-      <c r="H11" s="127">
-        <f>SUM(H4:H10)</f>
-        <v/>
-      </c>
-      <c r="I11" s="127">
-        <f>SUM(I4:I10)</f>
-        <v/>
-      </c>
-      <c r="J11" s="129" t="n"/>
-    </row>
+      <c r="G8" s="127">
+        <f>SUM(G4:G7)</f>
+        <v/>
+      </c>
+      <c r="H8" s="127">
+        <f>SUM(H4:H7)</f>
+        <v/>
+      </c>
+      <c r="I8" s="127">
+        <f>SUM(I4:I7)</f>
+        <v/>
+      </c>
+      <c r="J8" s="129" t="n"/>
+    </row>
+    <row r="9" ht="16.15" customHeight="1" thickTop="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
BKK layout: TIFFA (LCH54) in BMTP's slot, BMTP + new SCT (LCHY4) below BC2
Per sirichai 2026-10-12: TIFFA = LCH54 takes row 7 (and 34/48 in the
booking blocks); BMTP (BKKY4) moves below BC2 and SCT = LCHY4 goes under
it (template rows 10-11, 37-38, 51-52, restyled from the old BMTP row).
Applies to FULL INBOUND, CURRENT STOCK and BOOKING; dashboard follows
BKK_GROUPS. Note: LCH54 bookings were previously dropped (unmapped) and
now count, so TIFFA shows as short on 22GP in the 10-12 report.
Re-built 2026-10-12.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/(HAL)Stock form.xlsx
+++ b/(HAL)Stock form.xlsx
@@ -2640,12 +2640,12 @@
       <c r="AO6" s="30" t="n"/>
     </row>
     <row r="7" ht="15" customFormat="1" customHeight="1" s="34">
-      <c r="A7" s="136" t="inlineStr">
-        <is>
-          <t>BMTP</t>
-        </is>
-      </c>
-      <c r="B7" s="137" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>TIFFA</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>ICD</t>
         </is>
@@ -2659,15 +2659,15 @@
       <c r="I7" s="28" t="n"/>
       <c r="J7" s="28" t="n"/>
       <c r="K7" s="42" t="n"/>
-      <c r="L7" s="31" t="n"/>
-      <c r="M7" s="32" t="n"/>
-      <c r="N7" s="32" t="n"/>
-      <c r="O7" s="28" t="n"/>
-      <c r="P7" s="28" t="n"/>
-      <c r="Q7" s="28" t="n"/>
-      <c r="R7" s="28" t="n"/>
-      <c r="S7" s="28" t="n"/>
-      <c r="T7" s="33" t="n"/>
+      <c r="L7" s="23" t="n"/>
+      <c r="M7" s="28" t="n"/>
+      <c r="N7" s="28" t="n"/>
+      <c r="O7" s="29" t="n"/>
+      <c r="P7" s="29" t="n"/>
+      <c r="Q7" s="29" t="n"/>
+      <c r="R7" s="29" t="n"/>
+      <c r="S7" s="29" t="n"/>
+      <c r="T7" s="30" t="n"/>
       <c r="V7" s="23" t="inlineStr">
         <is>
           <t>HPT</t>
@@ -2814,8 +2814,16 @@
       <c r="AO9" s="30" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="35" t="n"/>
-      <c r="B10" s="36" t="n"/>
+      <c r="A10" s="136" t="inlineStr">
+        <is>
+          <t>BMTP</t>
+        </is>
+      </c>
+      <c r="B10" s="137" t="inlineStr">
+        <is>
+          <t>ICD</t>
+        </is>
+      </c>
       <c r="C10" s="41" t="n"/>
       <c r="D10" s="28" t="n"/>
       <c r="E10" s="28" t="n"/>
@@ -2825,15 +2833,15 @@
       <c r="I10" s="28" t="n"/>
       <c r="J10" s="28" t="n"/>
       <c r="K10" s="42" t="n"/>
-      <c r="L10" s="35" t="n"/>
-      <c r="M10" s="29" t="n"/>
-      <c r="N10" s="29" t="n"/>
-      <c r="O10" s="29" t="n"/>
-      <c r="P10" s="29" t="n"/>
-      <c r="Q10" s="29" t="n"/>
-      <c r="R10" s="29" t="n"/>
-      <c r="S10" s="29" t="n"/>
-      <c r="T10" s="30" t="n"/>
+      <c r="L10" s="31" t="n"/>
+      <c r="M10" s="32" t="n"/>
+      <c r="N10" s="32" t="n"/>
+      <c r="O10" s="28" t="n"/>
+      <c r="P10" s="28" t="n"/>
+      <c r="Q10" s="28" t="n"/>
+      <c r="R10" s="28" t="n"/>
+      <c r="S10" s="28" t="n"/>
+      <c r="T10" s="33" t="n"/>
       <c r="V10" s="35" t="inlineStr">
         <is>
           <t>PW</t>
@@ -2864,8 +2872,16 @@
       <c r="AO10" s="30" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="43" t="n"/>
-      <c r="B11" s="44" t="n"/>
+      <c r="A11" s="136" t="inlineStr">
+        <is>
+          <t>SCT</t>
+        </is>
+      </c>
+      <c r="B11" s="137" t="inlineStr">
+        <is>
+          <t>ICD</t>
+        </is>
+      </c>
       <c r="C11" s="41" t="n"/>
       <c r="D11" s="28" t="n"/>
       <c r="E11" s="28" t="n"/>
@@ -2875,15 +2891,15 @@
       <c r="I11" s="28" t="n"/>
       <c r="J11" s="28" t="n"/>
       <c r="K11" s="42" t="n"/>
-      <c r="L11" s="35" t="n"/>
-      <c r="M11" s="29" t="n"/>
-      <c r="N11" s="29" t="n"/>
-      <c r="O11" s="29" t="n"/>
-      <c r="P11" s="29" t="n"/>
-      <c r="Q11" s="29" t="n"/>
-      <c r="R11" s="29" t="n"/>
-      <c r="S11" s="29" t="n"/>
-      <c r="T11" s="30" t="n"/>
+      <c r="L11" s="31" t="n"/>
+      <c r="M11" s="32" t="n"/>
+      <c r="N11" s="32" t="n"/>
+      <c r="O11" s="28" t="n"/>
+      <c r="P11" s="28" t="n"/>
+      <c r="Q11" s="28" t="n"/>
+      <c r="R11" s="28" t="n"/>
+      <c r="S11" s="28" t="n"/>
+      <c r="T11" s="33" t="n"/>
       <c r="V11" s="35" t="n"/>
       <c r="W11" s="36" t="n"/>
       <c r="X11" s="39" t="n"/>
@@ -4290,25 +4306,25 @@
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="136" t="inlineStr">
-        <is>
-          <t>BMTP</t>
-        </is>
-      </c>
-      <c r="B34" s="137" t="inlineStr">
+      <c r="A34" s="23" t="inlineStr">
+        <is>
+          <t>TIFFA</t>
+        </is>
+      </c>
+      <c r="B34" s="44" t="inlineStr">
         <is>
           <t>ICD</t>
         </is>
       </c>
-      <c r="C34" s="25" t="n"/>
-      <c r="D34" s="26" t="n"/>
-      <c r="E34" s="26" t="n"/>
-      <c r="F34" s="26" t="n"/>
-      <c r="G34" s="26" t="n"/>
-      <c r="H34" s="94" t="n"/>
-      <c r="I34" s="38" t="n"/>
-      <c r="J34" s="38" t="n"/>
-      <c r="K34" s="83" t="n"/>
+      <c r="C34" s="41" t="n"/>
+      <c r="D34" s="28" t="n"/>
+      <c r="E34" s="28" t="n"/>
+      <c r="F34" s="28" t="n"/>
+      <c r="G34" s="28" t="n"/>
+      <c r="H34" s="32" t="n"/>
+      <c r="I34" s="49" t="n"/>
+      <c r="J34" s="49" t="n"/>
+      <c r="K34" s="82" t="n"/>
       <c r="L34" s="35">
         <f>SUM(L7-C34)</f>
         <v/>
@@ -4626,17 +4642,25 @@
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="43" t="n"/>
-      <c r="B37" s="44" t="n"/>
-      <c r="C37" s="48" t="n"/>
-      <c r="D37" s="49" t="n"/>
-      <c r="E37" s="49" t="n"/>
-      <c r="F37" s="49" t="n"/>
-      <c r="G37" s="49" t="n"/>
-      <c r="H37" s="49" t="n"/>
-      <c r="I37" s="49" t="n"/>
-      <c r="J37" s="49" t="n"/>
-      <c r="K37" s="82" t="n"/>
+      <c r="A37" s="136" t="inlineStr">
+        <is>
+          <t>BMTP</t>
+        </is>
+      </c>
+      <c r="B37" s="137" t="inlineStr">
+        <is>
+          <t>ICD</t>
+        </is>
+      </c>
+      <c r="C37" s="25" t="n"/>
+      <c r="D37" s="26" t="n"/>
+      <c r="E37" s="26" t="n"/>
+      <c r="F37" s="26" t="n"/>
+      <c r="G37" s="26" t="n"/>
+      <c r="H37" s="94" t="n"/>
+      <c r="I37" s="38" t="n"/>
+      <c r="J37" s="38" t="n"/>
+      <c r="K37" s="83" t="n"/>
       <c r="L37" s="35">
         <f>SUM(L10-C37)</f>
         <v/>
@@ -4730,17 +4754,25 @@
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="43" t="n"/>
-      <c r="B38" s="44" t="n"/>
-      <c r="C38" s="48" t="n"/>
-      <c r="D38" s="49" t="n"/>
-      <c r="E38" s="49" t="n"/>
-      <c r="F38" s="49" t="n"/>
-      <c r="G38" s="49" t="n"/>
-      <c r="H38" s="49" t="n"/>
-      <c r="I38" s="49" t="n"/>
-      <c r="J38" s="49" t="n"/>
-      <c r="K38" s="82" t="n"/>
+      <c r="A38" s="136" t="inlineStr">
+        <is>
+          <t>SCT</t>
+        </is>
+      </c>
+      <c r="B38" s="137" t="inlineStr">
+        <is>
+          <t>ICD</t>
+        </is>
+      </c>
+      <c r="C38" s="25" t="n"/>
+      <c r="D38" s="26" t="n"/>
+      <c r="E38" s="26" t="n"/>
+      <c r="F38" s="26" t="n"/>
+      <c r="G38" s="26" t="n"/>
+      <c r="H38" s="94" t="n"/>
+      <c r="I38" s="38" t="n"/>
+      <c r="J38" s="38" t="n"/>
+      <c r="K38" s="83" t="n"/>
       <c r="L38" s="35">
         <f>SUM(L11-C38)</f>
         <v/>
@@ -5788,25 +5820,25 @@
       </c>
     </row>
     <row r="48" ht="15" customHeight="1">
-      <c r="A48" s="136" t="inlineStr">
-        <is>
-          <t>BMTP</t>
-        </is>
-      </c>
-      <c r="B48" s="137" t="inlineStr">
+      <c r="A48" s="23" t="inlineStr">
+        <is>
+          <t>TIFFA</t>
+        </is>
+      </c>
+      <c r="B48" s="44" t="inlineStr">
         <is>
           <t>ICD</t>
         </is>
       </c>
-      <c r="C48" s="25" t="n"/>
-      <c r="D48" s="26" t="n"/>
-      <c r="E48" s="26" t="n"/>
-      <c r="F48" s="26" t="n"/>
-      <c r="G48" s="26" t="n"/>
-      <c r="H48" s="26" t="n"/>
-      <c r="I48" s="26" t="n"/>
-      <c r="J48" s="26" t="n"/>
-      <c r="K48" s="27" t="n"/>
+      <c r="C48" s="41" t="n"/>
+      <c r="D48" s="28" t="n"/>
+      <c r="E48" s="28" t="n"/>
+      <c r="F48" s="28" t="n"/>
+      <c r="G48" s="28" t="n"/>
+      <c r="H48" s="28" t="n"/>
+      <c r="I48" s="28" t="n"/>
+      <c r="J48" s="28" t="n"/>
+      <c r="K48" s="42" t="n"/>
       <c r="L48" s="35">
         <f>SUM(L34-C48)</f>
         <v/>
@@ -6124,17 +6156,25 @@
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
-      <c r="A51" s="43" t="n"/>
-      <c r="B51" s="44" t="n"/>
-      <c r="C51" s="41" t="n"/>
-      <c r="D51" s="28" t="n"/>
-      <c r="E51" s="28" t="n"/>
-      <c r="F51" s="28" t="n"/>
-      <c r="G51" s="28" t="n"/>
-      <c r="H51" s="28" t="n"/>
-      <c r="I51" s="28" t="n"/>
-      <c r="J51" s="28" t="n"/>
-      <c r="K51" s="42" t="n"/>
+      <c r="A51" s="136" t="inlineStr">
+        <is>
+          <t>BMTP</t>
+        </is>
+      </c>
+      <c r="B51" s="137" t="inlineStr">
+        <is>
+          <t>ICD</t>
+        </is>
+      </c>
+      <c r="C51" s="25" t="n"/>
+      <c r="D51" s="26" t="n"/>
+      <c r="E51" s="26" t="n"/>
+      <c r="F51" s="26" t="n"/>
+      <c r="G51" s="26" t="n"/>
+      <c r="H51" s="26" t="n"/>
+      <c r="I51" s="26" t="n"/>
+      <c r="J51" s="26" t="n"/>
+      <c r="K51" s="27" t="n"/>
       <c r="L51" s="35">
         <f>SUM(L37-C51)</f>
         <v/>
@@ -6228,17 +6268,25 @@
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
-      <c r="A52" s="43" t="n"/>
-      <c r="B52" s="44" t="n"/>
-      <c r="C52" s="41" t="n"/>
-      <c r="D52" s="28" t="n"/>
-      <c r="E52" s="28" t="n"/>
-      <c r="F52" s="28" t="n"/>
-      <c r="G52" s="28" t="n"/>
-      <c r="H52" s="28" t="n"/>
-      <c r="I52" s="28" t="n"/>
-      <c r="J52" s="28" t="n"/>
-      <c r="K52" s="42" t="n"/>
+      <c r="A52" s="136" t="inlineStr">
+        <is>
+          <t>SCT</t>
+        </is>
+      </c>
+      <c r="B52" s="137" t="inlineStr">
+        <is>
+          <t>ICD</t>
+        </is>
+      </c>
+      <c r="C52" s="25" t="n"/>
+      <c r="D52" s="26" t="n"/>
+      <c r="E52" s="26" t="n"/>
+      <c r="F52" s="26" t="n"/>
+      <c r="G52" s="26" t="n"/>
+      <c r="H52" s="26" t="n"/>
+      <c r="I52" s="26" t="n"/>
+      <c r="J52" s="26" t="n"/>
+      <c r="K52" s="27" t="n"/>
       <c r="L52" s="35">
         <f>SUM(L38-C52)</f>
         <v/>
@@ -6706,8 +6754,8 @@
   <mergeCells count="46">
     <mergeCell ref="V55:W55"/>
     <mergeCell ref="W59:AO59"/>
+    <mergeCell ref="A15:B15"/>
     <mergeCell ref="AG2:AL2"/>
-    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A2:B3"/>
     <mergeCell ref="W58:AO58"/>
     <mergeCell ref="I43:K43"/>

</xml_diff>